<commit_message>
feat(night-r4): integrate 10 agent branches — 5 tools (Capability/Ambition/Focus/Narrative/Risk → 19/19) + RAID handoff, maturity path N→N+1 (DRD/SIRI/ADMA), finance O4.5-4.7 (WACC/statements/post-mortem), 3 doc-editors on Editor Shell, 9 hubs c.* tokens, premium PPTX/XLSX stylers, generic Tools→Inicjatywy handoff, M15↔M16 reconciliation + M06 routing fix
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/deliverables/runs/ATELIER-TABLE.xlsx
+++ b/docs/qa/deliverables/runs/ATELIER-TABLE.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="102">
   <si>
     <t>Priority</t>
   </si>
@@ -112,6 +112,9 @@
     <t>Gap severity (0-100)</t>
   </si>
   <si>
+    <t>Health</t>
+  </si>
+  <si>
     <t>Line 3 OEE</t>
   </si>
   <si>
@@ -139,6 +142,9 @@
     <t>War-room + escalation</t>
   </si>
   <si>
+    <t>In Progress</t>
+  </si>
+  <si>
     <t>Repeat defect rate</t>
   </si>
   <si>
@@ -164,6 +170,12 @@
   </si>
   <si>
     <t>8-10 min</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>US requirement</t>
@@ -318,7 +330,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.##"/>
     <numFmt numFmtId="165" formatCode="# ##0.00&quot; zł&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -329,6 +341,20 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF85182F"/>
+    </font>
+    <font>
+      <color rgb="FF9A6A00"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1D7A54"/>
+    </font>
+    <font>
+      <b/>
     </font>
     <font>
       <b/>
@@ -353,7 +379,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -372,11 +398,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4F4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF1B5FA8"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -388,14 +429,25 @@
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
-      <bottom style="thin"/>
+      <bottom style="medium">
+        <color rgb="FF1D9E75"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF64748B"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -418,16 +470,34 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1065,17 +1135,18 @@
   <sheetPr>
     <tabColor rgb="FF1D9E75"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="3" width="23" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -1094,16 +1165,19 @@
       <c r="F1" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="4">
         <v>2.4</v>
@@ -1114,16 +1188,19 @@
       <c r="F2" s="2">
         <v>82</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D3" s="7">
         <v>4</v>
@@ -1134,16 +1211,19 @@
       <c r="F3" s="5">
         <v>90</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D4" s="4">
         <v>2</v>
@@ -1154,16 +1234,19 @@
       <c r="F4" s="2">
         <v>74</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D5" s="7">
         <v>0.9</v>
@@ -1174,16 +1257,19 @@
       <c r="F5" s="5">
         <v>68</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D6" s="4">
         <v>2</v>
@@ -1194,16 +1280,19 @@
       <c r="F6" s="2">
         <v>66</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D7" s="7">
         <v>0.6</v>
@@ -1214,9 +1303,35 @@
       <c r="F7" s="5">
         <v>60</v>
       </c>
+      <c r="G7" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="12">
+        <f>SUM(D2:D7)</f>
+      </c>
+      <c r="E8" s="12">
+        <f>SUM(E2:E7)</f>
+      </c>
+      <c r="F8" s="13">
+        <f>ROUND(AVERAGE(F2:F7),0)</f>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>53</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F7">
+  <conditionalFormatting sqref="F2:F8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1248,83 +1363,83 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>20</v>
@@ -1332,13 +1447,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>12</v>
@@ -1346,58 +1461,58 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1430,63 +1545,63 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="8"/>
+      <c r="A1" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="14"/>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B2" s="9"/>
+      <c r="A2" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="15"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>87</v>
+      <c r="A4" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>89</v>
+      <c r="A5" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>91</v>
+      <c r="A6" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>93</v>
+      <c r="A7" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>95</v>
+      <c r="A8" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>97</v>
+      <c r="A9" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>